<commit_message>
update de acuerdos de cartera inteligente
</commit_message>
<xml_diff>
--- a/agreement_report.xlsx
+++ b/agreement_report.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{BF0413D3-08C4-46CF-B91C-B7F1DE8BE3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADC9A750-3E59-46CC-843A-99C2110A66F1}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{F34F9A79-B068-42F3-8507-C40FB81D6044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB4C8FF3-52E4-4B81-B292-9995E8B2E0AC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -36,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="192">
   <si>
     <t>Reporte de Acuerdos</t>
   </si>
@@ -152,6 +149,9 @@
     <t>ANA MARIA</t>
   </si>
   <si>
+    <t>Se han dado conversaciones y se ha analizado como propuesta una modificación legislativa que permitiría presupuestar la donación de manera similar a un préstamo. El Banco está a la espera de que inicie formalmente el trámite legislativo de la propuesta.</t>
+  </si>
+  <si>
     <t>30/nov/2026</t>
   </si>
   <si>
@@ -170,139 +170,361 @@
     <t>Vigente</t>
   </si>
   <si>
+    <t>Ejecución de productos claves/Ruta crítica</t>
+  </si>
+  <si>
+    <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados (Fuente BID).</t>
+  </si>
+  <si>
+    <t>Debe definirse para iniciar y completar el producto oportunamente.</t>
+  </si>
+  <si>
+    <t>Planificación de proyectos</t>
+  </si>
+  <si>
+    <t>Identificación, duración y secuenciación de tareas.</t>
+  </si>
+  <si>
+    <t>El OE comunicará formalmente al MH/ DGGDP y al Banco el proyecto escogido para la estructuración del 2ndo proyecto APP antes del 31 de agosto de 2026, considerando las necesidades de recurso humano requerida para su revisión</t>
+  </si>
+  <si>
+    <t>31/ago/2026</t>
+  </si>
+  <si>
+    <t>MARIANO ANSALDO</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>CR-L1137</t>
+  </si>
+  <si>
+    <t>4871/OC-CR</t>
+  </si>
+  <si>
+    <t>CIS</t>
+  </si>
+  <si>
+    <t>Programa de Seguridad Ciudadana y Prevención de Violencia</t>
+  </si>
+  <si>
+    <t>Alcance/Cumplimiento de la Matriz de Resultados</t>
+  </si>
+  <si>
+    <t>Al ser obras multiples, se debe actualizar el calculo de la linea base y meta para los indicadores con base en el los productos efectivamente ejecutados por la operacion</t>
+  </si>
+  <si>
+    <t>Diseño técnico</t>
+  </si>
+  <si>
+    <t>Evaluación de eficiencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El OE formalizará el cambio de medición de los indicadores con base en los distritos intervenidos antes de 31 de julio, asegurando que en la próxima reunión de cartera se visualicen los datos. </t>
+  </si>
+  <si>
+    <t>31/jul/2026</t>
+  </si>
+  <si>
+    <t>NORMA CONSTANZA</t>
+  </si>
+  <si>
+    <t>Se presentó la memoria de cálculo y propuesta de modificación de indicadores, la cual está en revisión del banco para formalizarla.</t>
+  </si>
+  <si>
+    <t>Facilitar y documentar la medicion de indicadores y sustituir indicadores que no pueden medirse.</t>
+  </si>
+  <si>
+    <t>Estrategia de monitoreo y evaluación</t>
+  </si>
+  <si>
+    <t>Calidad de los indicadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El OE y el Banco acordarán una metodología de medición de indicadores (fuente, responsable y cálculo), actividades necesarias para realizar las mediciones y definir un sustituto para indicador de resultado 1.2 (reacciones xenófobas en tweets). </t>
+  </si>
+  <si>
+    <t>15/oct/2026</t>
+  </si>
+  <si>
+    <t>En la misión de julio 2026 se definieron líneas de acción para esta propuesta, pero aun se encuentra en proceso.</t>
+  </si>
+  <si>
+    <t>CR-L1157</t>
+  </si>
+  <si>
+    <t>6061/OC-CR</t>
+  </si>
+  <si>
+    <t>ENE</t>
+  </si>
+  <si>
+    <t>Segundo Programa de Energía Renovable, Transmisión y Distribución de Electricidad</t>
+  </si>
+  <si>
+    <t>Los cambios deben tramitarse como una solicitud de modificacion del contrato con apoyo del garante del prestamo.</t>
+  </si>
+  <si>
+    <t>Legislación y regulación</t>
+  </si>
+  <si>
+    <t>Procesos legales y regulatorios</t>
+  </si>
+  <si>
+    <t>Ante la necesidad de sustitución de productos con recursos del crédito, el ICE analizará el mecanismo para formalizar los cambios al contrato de préstamo y elaborará la documentación respectiva.</t>
+  </si>
+  <si>
+    <t>14/ago/2026</t>
+  </si>
+  <si>
+    <t>EDWIN ORLANDO</t>
+  </si>
+  <si>
+    <t>Se identificó la posibilidad de incorporar una modificación de montos entre categorías de inversión como parte de los cambios contractuales que podría formalizar el ICE. Por lo anterior, se decide trasladar a finales de diciembre el proceso de formalización de cambios para contar con los montos de ofertas realmente recibidas de productos del componente 1.</t>
+  </si>
+  <si>
+    <t>CR-L1156</t>
+  </si>
+  <si>
+    <t>6017/OC-CR</t>
+  </si>
+  <si>
+    <t>SPL</t>
+  </si>
+  <si>
+    <t>Apoyo al fortalecimiento y expansión del sistema nacional de cuidados de Costa Rica</t>
+  </si>
+  <si>
+    <t>Elegibilidad pendiente</t>
+  </si>
+  <si>
+    <t>en coordinación con el Ministerio de Hacienda, quien orientará al Banco respecto a los plazos para su cumplimiento de la elegibilidad</t>
+  </si>
+  <si>
+    <t>El Banco dará seguimiento al cumplimiento de las condiciones establecidas en el Artículo 4.01 del Contrato de Préstamo (informe jurídico, firmas autorizadas y cuenta bancaria especial), así como a la vigencia del IAMC.</t>
+  </si>
+  <si>
+    <t>15/dic/2026</t>
+  </si>
+  <si>
+    <t>PATRICIA CAROLINA</t>
+  </si>
+  <si>
+    <t>CR-L1032</t>
+  </si>
+  <si>
+    <t>3071/OC-CR</t>
+  </si>
+  <si>
+    <t>Programa de Infraestructura de Transporte (PIT)</t>
+  </si>
+  <si>
+    <t>Cumplidos</t>
+  </si>
+  <si>
+    <t>Recopilación de datos e informes</t>
+  </si>
+  <si>
+    <t>El MOPT informará al Ministerio de Hacienda y al Banco sobre los avances en el proceso de ejecución de obras de la sección Barranca-Limonal</t>
+  </si>
+  <si>
+    <t>30/sep/2026</t>
+  </si>
+  <si>
+    <t>La Unidad Ejecutora concluirá el plan de mediciones de resultados de proyectos concluidos antes de la finalización del plazo actual de desembolsos.</t>
+  </si>
+  <si>
+    <t>13/nov/2026</t>
+  </si>
+  <si>
+    <t>La Unidad Ejecutora programará mediciones parciales de los indicadores de resultados del Programa asociadas con Barranca  Limonal y la Angostura en fechas que serán definidas mediante un cronograma a ser presentado por el MOPT al BID con copia al MH</t>
+  </si>
+  <si>
+    <t>Plazo de desembolsos vencido o próximo a vencer</t>
+  </si>
+  <si>
+    <t>Plazo de desembolsos próximo a vencer</t>
+  </si>
+  <si>
+    <t>Compromiso y coordinación</t>
+  </si>
+  <si>
+    <t>Relaciones intergubernamentales e intragubernamentales</t>
+  </si>
+  <si>
+    <t>La UEP del PIT elaborará un análisis financiero que evalúe escenarios contractuales vis a vis, implicando la decisión de continuidad o no de contratos del gestor, en el marco de la decisión de extensión o no del plazo de desembolsos....</t>
+  </si>
+  <si>
+    <t>01/jul/2026</t>
+  </si>
+  <si>
+    <t>La UEP ha presentado la información y ahora corresponde al MH y al Banco definir las condiciones para la posible extensión</t>
+  </si>
+  <si>
+    <t>CR-L1151</t>
+  </si>
+  <si>
+    <t>5823/OC-CR</t>
+  </si>
+  <si>
+    <t>Programa de Infraestructura Vial y Movilidad Urbana: conectividad resiliente</t>
+  </si>
+  <si>
+    <t>Gobernanza pública y política</t>
+  </si>
+  <si>
+    <t>Agenda política</t>
+  </si>
+  <si>
+    <t>El OE definirá los montos y fuentes de financiamiento necesarios para asegurar la ejecución del 100% de la RN 35 cumpliendo los compromisos del Contrato de Préstamo, incluyendo las decisiones sobre proceso de adquisición del Tramo Central.</t>
+  </si>
+  <si>
+    <t>15/sep/2026</t>
+  </si>
+  <si>
+    <t>Actualmente se encuentra en revisión una extensión al PROGRAMA CR-L1032 para también asegurar una fuente de financiamiento que sea suficiente para la ejecución de cualquier ajuste en el Programa.</t>
+  </si>
+  <si>
+    <t>Ritmo de la ejecución financiera</t>
+  </si>
+  <si>
+    <t>Capacidad organizacional</t>
+  </si>
+  <si>
+    <t>Procesos y Sistemas</t>
+  </si>
+  <si>
+    <t>Valoración por parte del Organismo Ejecutor del plan de trabajo y de las alertas tempranas para priorizar la ejecución de los recursos correspondientes a la fuente de financiamiento 3072/CH-CR antes de su fecha de último desembolso (nov/2026).</t>
+  </si>
+  <si>
+    <t>12/nov/2026</t>
+  </si>
+  <si>
+    <t>CR-L1065</t>
+  </si>
+  <si>
+    <t>4507/OC-CR</t>
+  </si>
+  <si>
+    <t>Programa Red Vial Cantonal II</t>
+  </si>
+  <si>
+    <t>Anticipos pendientes de rendición</t>
+  </si>
+  <si>
+    <t>Caminos cantonales rehabilitados. Puentes construidos o rehabilitados</t>
+  </si>
+  <si>
+    <t>Ambiente económico</t>
+  </si>
+  <si>
+    <t>Precio de bienes y servicios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Organismo Ejecutor (OE) debe presentar al Banco detalle de justificación parcial de gastos con corte al 30 de abril 2026, lo cual permitirá pronosticar cómo cerrará la operación y si se debe o no debe hacerse devolución de fondos al BID. </t>
+  </si>
+  <si>
+    <t>30/may/2026</t>
+  </si>
+  <si>
+    <t>La justificación indicada fue presentada. El OE con la ampliación al plazo de cierre otorgado por el BID, presentaría la última justificación del Programa con corte al 15 de setiembre.</t>
+  </si>
+  <si>
+    <t>Cálculo de costo</t>
+  </si>
+  <si>
+    <t>Sostener reuniones de seguimiento orientadas al cierre técnico, financiero y administrativo previsto para el del 24 de julio. La primera reunión se realizará el 28 de mayo 2026.</t>
+  </si>
+  <si>
+    <t>24/jul/2026</t>
+  </si>
+  <si>
+    <t>Las reuniones de seguimiento se han realizado y la última se llevará a cabo el a más tardar el 14 de setiembre.</t>
+  </si>
+  <si>
+    <t>El pago permitirá dar cumplimiento a pasivos socioambientales del proyecto</t>
+  </si>
+  <si>
+    <t>El OE debe dar seguimiento en la Asamblea Legislativa al trámite de aprobación del Presupuesto Extraordinario (recursos para indemnización). Para asegurar el pago de los montos acordados de indemnización en el caso Quebrada Mina.</t>
+  </si>
+  <si>
+    <t>Cumplido. La Ley de presupuesto extraordinario fue aprobada por la Asamblea Legislativa y el pago realizado por parte del MOPT con cargo al Programa.</t>
+  </si>
+  <si>
     <t>Retrasos en el cronograma</t>
   </si>
   <si>
     <t xml:space="preserve">la reprogramacion de la operación permitirá conocer la fecha de fin estimada para el plazo de desembolsos. </t>
   </si>
   <si>
-    <t>Planificación de proyectos</t>
-  </si>
-  <si>
-    <t>Identificación, duración y secuenciación de tareas.</t>
-  </si>
-  <si>
     <t>Actualizar el Plan de Ejecución del Programa para identificar la ruta crítica vigente y anticipar la estrategia de ejecución conforme la fecha vigente y la proyectada para la fecha de último desembolso.</t>
   </si>
   <si>
-    <t>13/nov/2026</t>
-  </si>
-  <si>
-    <t>MARIANO ANSALDO</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Ejecución de productos claves/Ruta crítica</t>
-  </si>
-  <si>
-    <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados (Fuente BID).</t>
-  </si>
-  <si>
-    <t>Debe definirse para iniciar y completar el producto oportunamente.</t>
-  </si>
-  <si>
-    <t>El OE comunicará formalmente al MH/ DGGDP y al Banco el proyecto escogido para la estructuración del 2ndo proyecto APP antes del 31 de agosto de 2026, considerando las necesidades de recurso humano requerida para su revisión</t>
-  </si>
-  <si>
-    <t>31/ago/2026</t>
-  </si>
-  <si>
-    <t>CR-L1137</t>
-  </si>
-  <si>
-    <t>4871/OC-CR</t>
-  </si>
-  <si>
-    <t>CIS</t>
-  </si>
-  <si>
-    <t>Programa de Seguridad Ciudadana y Prevención de Violencia</t>
-  </si>
-  <si>
-    <t>Alcance/Cumplimiento de la Matriz de Resultados</t>
-  </si>
-  <si>
-    <t>Al ser obras multiples, se debe actualizar el calculo de la linea base y meta para los indicadores con base en el los productos efectivamente ejecutados por la operacion</t>
-  </si>
-  <si>
-    <t>Diseño técnico</t>
-  </si>
-  <si>
-    <t>Evaluación de eficiencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El OE formalizará el cambio de medición de los indicadores con base en los distritos intervenidos antes de 31 de julio, asegurando que en la próxima reunión de cartera se visualicen los datos. </t>
-  </si>
-  <si>
-    <t>31/jul/2026</t>
-  </si>
-  <si>
-    <t>NORMA CONSTANZA</t>
-  </si>
-  <si>
-    <t>Facilitar y documentar la medicion de indicadores y sustituir indicadores que no pueden medirse.</t>
-  </si>
-  <si>
-    <t>Estrategia de monitoreo y evaluación</t>
-  </si>
-  <si>
-    <t>Calidad de los indicadores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El OE y el Banco acordarán una metodología de medición de indicadores (fuente, responsable y cálculo), actividades necesarias para realizar las mediciones y definir un sustituto para indicador de resultado 1.2 (reacciones xenófobas en tweets). </t>
-  </si>
-  <si>
-    <t>15/oct/2026</t>
-  </si>
-  <si>
-    <t>CR-L1157</t>
-  </si>
-  <si>
-    <t>6061/OC-CR</t>
-  </si>
-  <si>
-    <t>ENE</t>
-  </si>
-  <si>
-    <t>Segundo Programa de Energía Renovable, Transmisión y Distribución de Electricidad</t>
-  </si>
-  <si>
-    <t>Elegibilidad pendiente</t>
+    <t>Se entregó PEP actualziado en informe semestral y en reunión de seguimiento del 23 de octubre. En la RGC se presentará la ruta crítica.</t>
+  </si>
+  <si>
+    <t>Plan de Adquisiciones desactualizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estas obras deberán ejecutarse previo a la finalización del período de notificación de defectos de la obra principal en agosto de 2027, y contemplar un monto total que no exceda los recursos remanentes del proyecto. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El OE elaborará y entregará de forma coordinada al BID una estrategia de adquisiciones para las Obras No Sustanciales del proyecto TarasLa Lima (temas urbanísticos tácticos y paisajismos). </t>
+  </si>
+  <si>
+    <t>Establecer mecanismos de mitigacion de atrasos del programa ante los problemas de ejecución de contratistas de obras.</t>
+  </si>
+  <si>
+    <t>Tipo de cambio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El OE remitirá un diagnóstico que presente escenarios, estrategias financieras y posibles soluciones para los contratos de obra de los 4 Centros Cívicos por la Paz con baja ejecución </t>
+  </si>
+  <si>
+    <t>15/jul/2026</t>
+  </si>
+  <si>
+    <t>El diagnóstico se presentó, a la vez que se procedió a la cancelación anticipada de los contratos de obra por incumplimiento del contratista. Actualmente se encuentra en licitación los procesos para la conclusión de obras de los 4 centros cívicos.</t>
+  </si>
+  <si>
+    <t>Los atrasos en la ejecucion de proyectos han impedido alcanzar los desembolsos planeados y afecta la posibilidad de incorporar los recursos de ejecucion para el 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El OE evaluará la posibilidad de replantear la interpretación de las normas para incorporar los recursos de la donación de forma similar a los empréstitos. </t>
+  </si>
+  <si>
+    <t>30/jul/2026</t>
+  </si>
+  <si>
+    <t>Se realizó la evaluación. La conclusión del prestatario es que no existe posibilidad de interpretación de las normas que permita la incorporación de los recursos por lo que se procederá con un proyecto de modificación legislativa para lograrlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la misión deberá definir y formalizar el alcance de productos a financiar, estrategia de ejecución, estrategia de adquisiciones, cronograma detallado y evaluabilidad de resultados, y evaluar la necesidad y magnitud de una eventual extensión. </t>
+  </si>
+  <si>
+    <t>El OE, autoridades y el Banco coordinarán para realizar una misión de administración, posterior a la primera sesión del Comité Directivo, para definir y formalizar la reprogramacion de la operación.</t>
   </si>
   <si>
     <t>principales temas a resolver para la elegibilidad son: la formalizacion del manual de operaciones con detalle de los procesos internos y aportar el informe de control interno del ejecutor</t>
   </si>
   <si>
-    <t>Capacidad organizacional</t>
-  </si>
-  <si>
-    <t>Procesos y Sistemas</t>
-  </si>
-  <si>
     <t xml:space="preserve">El ICE ejecutará oportunamente el plan para obtener la elegibilidad. </t>
   </si>
   <si>
-    <t>15/jul/2026</t>
-  </si>
-  <si>
-    <t>EDWIN ORLANDO</t>
-  </si>
-  <si>
-    <t>Los cambios deben tramitarse como una solicitud de modificacion del contrato con apoyo del garante del prestamo.</t>
-  </si>
-  <si>
-    <t>Legislación y regulación</t>
-  </si>
-  <si>
-    <t>Procesos legales y regulatorios</t>
-  </si>
-  <si>
-    <t>Ante la necesidad de sustitución de productos con recursos del crédito, el ICE analizará el mecanismo para formalizar los cambios al contrato de préstamo y elaborará la documentación respectiva.</t>
-  </si>
-  <si>
-    <t>14/ago/2026</t>
+    <t>El ICE presentó al Banco toda la documentación para dar por cumplidas las cláusulas de elegibilidad. El Banco se encuentra en análisis de la documentación.</t>
+  </si>
+  <si>
+    <t>Los productos a sustituir los transformadores deben ser congruentes con la teoria de cambio y deben contar con datos disponibles para calcular la linea base y la meta</t>
+  </si>
+  <si>
+    <t>Disponibilidad de datos y líneas de base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El ICE con apoyo del Banco identificará los productos que sustituyen a los transformadores, asegurando que las licitaciones respectivas cumplan con las políticas del Banco y contribuyan al logro de los indicadores establecidos. </t>
+  </si>
+  <si>
+    <t>Se definieron los productos y los indicadores de resultado respectivos. En cuanto se firme la ayuda memoria del taller de arranque se procederá a formalizar los cambios en los sistemas del Banco.</t>
   </si>
   <si>
     <t>CR-L1152</t>
@@ -329,6 +551,15 @@
     <t>LUANA</t>
   </si>
   <si>
+    <t>Teoría del cambio</t>
+  </si>
+  <si>
+    <t>El Banco coordinará con el MEP la revisión de las fichas técnicas por parte del Ministro, con el propósito de identificar eventuales ajustes adicionales que deban incorporarse y ser abordados durante el taller de arranque.</t>
+  </si>
+  <si>
+    <t>Se ha trabajado con distintas direcciones del MEP para hacer los ajustes. Este proceso seguirá hasta que inicie la ejecución del programa</t>
+  </si>
+  <si>
     <t>Capacidad de la unidad ejecutora</t>
   </si>
   <si>
@@ -338,193 +569,7 @@
     <t>El Banco dará continuidad a las reuniones con direcciones técnicas para dar seguimiento al apoyo técnico, de cara al inicio de la ejecución del Programa.</t>
   </si>
   <si>
-    <t>15/dic/2026</t>
-  </si>
-  <si>
-    <t>CR-L1156</t>
-  </si>
-  <si>
-    <t>6017/OC-CR</t>
-  </si>
-  <si>
-    <t>SPL</t>
-  </si>
-  <si>
-    <t>Apoyo al fortalecimiento y expansión del sistema nacional de cuidados de Costa Rica</t>
-  </si>
-  <si>
-    <t>en coordinación con el Ministerio de Hacienda, quien orientará al Banco respecto a los plazos para su cumplimiento de la elegibilidad</t>
-  </si>
-  <si>
-    <t>El Banco dará seguimiento al cumplimiento de las condiciones establecidas en el Artículo 4.01 del Contrato de Préstamo (informe jurídico, firmas autorizadas y cuenta bancaria especial), así como a la vigencia del IAMC.</t>
-  </si>
-  <si>
-    <t>PATRICIA CAROLINA</t>
-  </si>
-  <si>
-    <t>CR-L1032</t>
-  </si>
-  <si>
-    <t>3071/OC-CR</t>
-  </si>
-  <si>
-    <t>Programa de Infraestructura de Transporte (PIT)</t>
-  </si>
-  <si>
-    <t>Cumplidos</t>
-  </si>
-  <si>
-    <t>Recopilación de datos e informes</t>
-  </si>
-  <si>
-    <t>El MOPT informará al Ministerio de Hacienda y al Banco sobre los avances en el proceso de ejecución de obras de la sección Barranca-Limonal</t>
-  </si>
-  <si>
-    <t>30/sep/2026</t>
-  </si>
-  <si>
-    <t>La Unidad Ejecutora concluirá el plan de mediciones de resultados de proyectos concluidos antes de la finalización del plazo actual de desembolsos.</t>
-  </si>
-  <si>
-    <t>La Unidad Ejecutora programará mediciones parciales de los indicadores de resultados del Programa asociadas con Barranca  Limonal y la Angostura en fechas que serán definidas mediante un cronograma a ser presentado por el MOPT al BID con copia al MH</t>
-  </si>
-  <si>
-    <t>Plazo de desembolsos vencido o próximo a vencer</t>
-  </si>
-  <si>
-    <t>Plazo de desembolsos próximo a vencer</t>
-  </si>
-  <si>
-    <t>Compromiso y coordinación</t>
-  </si>
-  <si>
-    <t>Relaciones intergubernamentales e intragubernamentales</t>
-  </si>
-  <si>
-    <t>La UEP del PIT elaborará un análisis financiero que evalúe escenarios contractuales vis a vis, implicando la decisión de continuidad o no de contratos del gestor, en el marco de la decisión de extensión o no del plazo de desembolsos....</t>
-  </si>
-  <si>
-    <t>01/jul/2026</t>
-  </si>
-  <si>
-    <t>CR-L1151</t>
-  </si>
-  <si>
-    <t>5823/OC-CR</t>
-  </si>
-  <si>
-    <t>Programa de Infraestructura Vial y Movilidad Urbana: conectividad resiliente</t>
-  </si>
-  <si>
-    <t>Gobernanza pública y política</t>
-  </si>
-  <si>
-    <t>Agenda política</t>
-  </si>
-  <si>
-    <t>El OE definirá los montos y fuentes de financiamiento necesarios para asegurar la ejecución del 100% de la RN 35 cumpliendo los compromisos del Contrato de Préstamo, incluyendo las decisiones sobre proceso de adquisición del Tramo Central.</t>
-  </si>
-  <si>
-    <t>15/sep/2026</t>
-  </si>
-  <si>
-    <t>Ritmo de la ejecución financiera</t>
-  </si>
-  <si>
-    <t>Valoración por parte del Organismo Ejecutor del plan de trabajo y de las alertas tempranas para priorizar la ejecución de los recursos correspondientes a la fuente de financiamiento 3072/CH-CR antes de su fecha de último desembolso (nov/2026).</t>
-  </si>
-  <si>
-    <t>12/nov/2026</t>
-  </si>
-  <si>
-    <t>CR-L1065</t>
-  </si>
-  <si>
-    <t>4507/OC-CR</t>
-  </si>
-  <si>
-    <t>Programa Red Vial Cantonal II</t>
-  </si>
-  <si>
-    <t>Anticipos pendientes de rendición</t>
-  </si>
-  <si>
-    <t>Caminos cantonales rehabilitados. Puentes construidos o rehabilitados</t>
-  </si>
-  <si>
-    <t>Ambiente económico</t>
-  </si>
-  <si>
-    <t>Precio de bienes y servicios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Organismo Ejecutor (OE) debe presentar al Banco detalle de justificación parcial de gastos con corte al 30 de abril 2026, lo cual permitirá pronosticar cómo cerrará la operación y si se debe o no debe hacerse devolución de fondos al BID. </t>
-  </si>
-  <si>
-    <t>30/may/2026</t>
-  </si>
-  <si>
-    <t>Cálculo de costo</t>
-  </si>
-  <si>
-    <t>Sostener reuniones de seguimiento orientadas al cierre técnico, financiero y administrativo previsto para el del 24 de julio. La primera reunión se realizará el 28 de mayo 2026.</t>
-  </si>
-  <si>
-    <t>24/jul/2026</t>
-  </si>
-  <si>
-    <t>El pago permitirá dar cumplimiento a pasivos socioambientales del proyecto</t>
-  </si>
-  <si>
-    <t>El OE debe dar seguimiento en la Asamblea Legislativa al trámite de aprobación del Presupuesto Extraordinario (recursos para indemnización). Para asegurar el pago de los montos acordados de indemnización en el caso Quebrada Mina.</t>
-  </si>
-  <si>
-    <t>Plan de Adquisiciones desactualizado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estas obras deberán ejecutarse previo a la finalización del período de notificación de defectos de la obra principal en agosto de 2027, y contemplar un monto total que no exceda los recursos remanentes del proyecto. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">El OE elaborará y entregará de forma coordinada al BID una estrategia de adquisiciones para las Obras No Sustanciales del proyecto TarasLa Lima (temas urbanísticos tácticos y paisajismos). </t>
-  </si>
-  <si>
-    <t>Establecer mecanismos de mitigacion de atrasos del programa ante los problemas de ejecución de contratistas de obras.</t>
-  </si>
-  <si>
-    <t>Tipo de cambio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El OE remitirá un diagnóstico que presente escenarios, estrategias financieras y posibles soluciones para los contratos de obra de los 4 Centros Cívicos por la Paz con baja ejecución </t>
-  </si>
-  <si>
-    <t>Los atrasos en la ejecucion de proyectos han impedido alcanzar los desembolsos planeados y afecta la posibilidad de incorporar los recursos de ejecucion para el 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El OE evaluará la posibilidad de replantear la interpretación de las normas para incorporar los recursos de la donación de forma similar a los empréstitos. </t>
-  </si>
-  <si>
-    <t>30/jul/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">la misión deberá definir y formalizar el alcance de productos a financiar, estrategia de ejecución, estrategia de adquisiciones, cronograma detallado y evaluabilidad de resultados, y evaluar la necesidad y magnitud de una eventual extensión. </t>
-  </si>
-  <si>
-    <t>El OE, autoridades y el Banco coordinarán para realizar una misión de administración, posterior a la primera sesión del Comité Directivo, para definir y formalizar la reprogramacion de la operación.</t>
-  </si>
-  <si>
-    <t>Los productos a sustituir los transformadores deben ser congruentes con la teoria de cambio y deben contar con datos disponibles para calcular la linea base y la meta</t>
-  </si>
-  <si>
-    <t>Disponibilidad de datos y líneas de base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El ICE con apoyo del Banco identificará los productos que sustituyen a los transformadores, asegurando que las licitaciones respectivas cumplan con las políticas del Banco y contribuyan al logro de los indicadores establecidos. </t>
-  </si>
-  <si>
-    <t>Teoría del cambio</t>
-  </si>
-  <si>
-    <t>El Banco coordinará con el MEP la revisión de las fichas técnicas por parte del Ministro, con el propósito de identificar eventuales ajustes adicionales que deban incorporarse y ser abordados durante el taller de arranque.</t>
+    <t>Se llevaron a cabo reuniones técnicas con las direcciones esoecíficas, a cargo de los componentes de la operación, para avanzar en la identificación de actividades y de ajustes que haya que implementar en el taller de arranque</t>
   </si>
   <si>
     <t xml:space="preserve">El organismo ejecutor deberá socializar con el Ministerio de Hacienda una carta borrador del acuerdo relativo al cumplimiento de políticas. </t>
@@ -563,31 +608,7 @@
     <t>Total acuerdos:</t>
   </si>
   <si>
-    <t>Se ha realizado acercamientos del viceministro de Justicia para avanzar en el tema y el Banco ha presentado documentación de contexto sobre el problema para facilitar la búsqueda de soluciones.</t>
-  </si>
-  <si>
-    <t>El ejecutor presentó una propuesta de actualización de los valores base y meta de los indicadores. Se encuentra en revisión por parte del equipo del Banco</t>
-  </si>
-  <si>
-    <t>No ha habido avances en la propuesta de la metodología por parte del Ejecutor.</t>
-  </si>
-  <si>
-    <t>La única condición de elegibilidad pendiente es la aprobación del MOP. Se espera cumplir el 6/oct dentro del plazo de 180 días.</t>
-  </si>
-  <si>
-    <t>El ICE ha identificado el mecanismo y se encuentra en proceso de elaboración de la documentación</t>
-  </si>
-  <si>
-    <t>El diagnóstico fue presentado y se propuso la terminación anticipada de los contratos y contratación de otro contratista para finalizar las obras. Los procesos de contratación se encuentran andando.</t>
-  </si>
-  <si>
-    <t>La posibilidad de interpretación de la norma fue descartada por las autoridades.</t>
-  </si>
-  <si>
-    <t>La misión de administración fue realizada durante el mes de julio. Sin embargo, algunos de los acuerdos aun no han sido aprobados por el Comité Directivo ni formalizados ante el Banco.</t>
-  </si>
-  <si>
-    <t>Los productos fueron identificados e incluidos en la ayuda memoria del taller de arranque. Actualmente se encuentra en el proceso de formalización de los cambios ante el Banco.</t>
+    <t>La misión se realizó en julio 2026. Sin embargo, algunos de los acuerdos aun no han sido aprobados por el Comité Directivo ni formalizados ante el Banco.</t>
   </si>
 </sst>
 </file>
@@ -606,45 +627,45 @@
       <sz val="18"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -981,23 +1002,23 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A2:Z44"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="1"/>
-    <col min="2" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" customWidth="1"/>
-    <col min="7" max="7" width="43.42578125" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" customWidth="1"/>
-    <col min="10" max="11" width="29.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" customWidth="1"/>
+    <col min="2" max="3" width="16.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.88671875" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" customWidth="1"/>
+    <col min="6" max="6" width="19.109375" customWidth="1"/>
+    <col min="7" max="7" width="43.44140625" customWidth="1"/>
+    <col min="8" max="8" width="20.88671875" customWidth="1"/>
+    <col min="9" max="9" width="24.109375" customWidth="1"/>
+    <col min="10" max="11" width="29.5546875" customWidth="1"/>
     <col min="12" max="12" width="42" customWidth="1"/>
     <col min="13" max="14" width="44" customWidth="1"/>
     <col min="15" max="15" width="62" customWidth="1"/>
-    <col min="16" max="16" width="21.7109375" customWidth="1"/>
-    <col min="17" max="17" width="32.28515625" customWidth="1"/>
-    <col min="18" max="19" width="39.5703125" customWidth="1"/>
+    <col min="16" max="16" width="21.77734375" customWidth="1"/>
+    <col min="17" max="17" width="32.21875" customWidth="1"/>
+    <col min="18" max="19" width="39.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:26" ht="45.75" customHeight="1">
@@ -1006,7 +1027,7 @@
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
     </row>
-    <row r="3" spans="1:26" ht="23.25">
+    <row r="3" spans="1:26" ht="22.8">
       <c r="B3" s="12" t="s">
         <v>0</v>
       </c>
@@ -1014,7 +1035,7 @@
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
     </row>
-    <row r="5" spans="1:26" ht="12.75">
+    <row r="5" spans="1:26" ht="13.2">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1025,7 +1046,7 @@
       <c r="E5" s="13"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:26" ht="12.75">
+    <row r="6" spans="1:26" ht="13.2">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1035,7 +1056,7 @@
       </c>
       <c r="E6" s="13"/>
     </row>
-    <row r="7" spans="1:26" ht="12.75">
+    <row r="7" spans="1:26" ht="13.2">
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
@@ -1045,7 +1066,7 @@
       </c>
       <c r="E7" s="11"/>
     </row>
-    <row r="8" spans="1:26" ht="12.75">
+    <row r="8" spans="1:26" ht="13.2">
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1055,7 +1076,7 @@
       </c>
       <c r="E8" s="11"/>
     </row>
-    <row r="10" spans="1:26" s="1" customFormat="1" ht="12.75">
+    <row r="10" spans="1:26" s="1" customFormat="1" ht="13.2">
       <c r="B10" s="4" t="s">
         <v>8</v>
       </c>
@@ -1156,10 +1177,10 @@
         <v>37</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>175</v>
+        <v>38</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
@@ -1171,10 +1192,10 @@
     </row>
     <row r="12" spans="1:26" ht="36" customHeight="1">
       <c r="B12" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>28</v>
@@ -1183,50 +1204,52 @@
         <v>5</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K12" s="6"/>
+        <v>45</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>46</v>
+      </c>
       <c r="L12" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="R12" s="6"/>
       <c r="S12" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="36" customHeight="1">
       <c r="B13" s="6" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>28</v>
@@ -1235,106 +1258,106 @@
         <v>5</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>53</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="K13" s="6"/>
       <c r="L13" s="6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R13" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="S13" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="36" customHeight="1">
       <c r="B14" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="K14" s="6"/>
       <c r="L14" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>176</v>
+        <v>71</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="36" customHeight="1">
       <c r="B15" s="6" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>28</v>
@@ -1343,52 +1366,52 @@
         <v>5</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K15" s="6"/>
       <c r="L15" s="6" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>177</v>
+        <v>82</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="36" customHeight="1">
       <c r="B16" s="6" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>28</v>
@@ -1397,52 +1420,50 @@
         <v>5</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="K16" s="6"/>
       <c r="L16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="N16" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M16" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="O16" s="6" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>178</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="R16" s="6"/>
       <c r="S16" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="2:19" ht="36" customHeight="1">
       <c r="B17" s="6" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>28</v>
@@ -1451,52 +1472,50 @@
         <v>5</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="R17" s="6" t="s">
-        <v>179</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="R17" s="6"/>
       <c r="S17" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="2:19" ht="36" customHeight="1">
       <c r="B18" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>28</v>
@@ -1505,50 +1524,50 @@
         <v>5</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="K18" s="6"/>
       <c r="L18" s="6" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="R18" s="6"/>
       <c r="S18" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="2:19" ht="36" customHeight="1">
       <c r="B19" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>28</v>
@@ -1557,102 +1576,104 @@
         <v>5</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="K19" s="6"/>
       <c r="L19" s="6" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="P19" s="6" t="s">
         <v>100</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="R19" s="6"/>
       <c r="S19" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="2:19" ht="36" customHeight="1">
       <c r="B20" s="6" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="C20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="J20" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="K20" s="6"/>
       <c r="L20" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="N20" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>106</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="R20" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>108</v>
+      </c>
       <c r="S20" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="2:19" ht="36" customHeight="1">
       <c r="B21" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>28</v>
@@ -1661,50 +1682,52 @@
         <v>5</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P21" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R21" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="S21" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="2:19" ht="36" customHeight="1">
       <c r="B22" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>28</v>
@@ -1713,50 +1736,50 @@
         <v>5</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="K22" s="6"/>
       <c r="L22" s="6" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>69</v>
+        <v>118</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>49</v>
+        <v>121</v>
       </c>
       <c r="Q22" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="R22" s="6"/>
       <c r="S22" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="2:19" ht="36" customHeight="1">
       <c r="B23" s="6" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>28</v>
@@ -1765,50 +1788,52 @@
         <v>5</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>61</v>
+        <v>125</v>
       </c>
       <c r="K23" s="6"/>
       <c r="L23" s="6" t="s">
-        <v>61</v>
+        <v>126</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>69</v>
+        <v>127</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="O23" s="6" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="P23" s="6" t="s">
-        <v>49</v>
+        <v>130</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R23" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R23" s="6" t="s">
+        <v>131</v>
+      </c>
       <c r="S23" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="2:19" ht="36" customHeight="1">
       <c r="B24" s="6" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>28</v>
@@ -1817,102 +1842,106 @@
         <v>5</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="K24" s="6"/>
       <c r="L24" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="Q24" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R24" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R24" s="6" t="s">
+        <v>135</v>
+      </c>
       <c r="S24" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="2:19" ht="36" customHeight="1">
       <c r="B25" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G25" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="H25" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>33</v>
       </c>
       <c r="K25" s="6"/>
       <c r="L25" s="6" t="s">
-        <v>33</v>
+        <v>136</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>126</v>
+        <v>77</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="O25" s="6" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="P25" s="6" t="s">
-        <v>129</v>
+        <v>63</v>
       </c>
       <c r="Q25" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R25" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R25" s="6" t="s">
+        <v>138</v>
+      </c>
       <c r="S25" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="2:19" ht="36" customHeight="1">
       <c r="B26" s="6" t="s">
-        <v>123</v>
+        <v>40</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>124</v>
+        <v>41</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>28</v>
@@ -1921,50 +1950,52 @@
         <v>5</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>125</v>
+        <v>43</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="K26" s="6"/>
       <c r="L26" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R26" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="R26" s="6" t="s">
+        <v>142</v>
+      </c>
       <c r="S26" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:19" ht="36" customHeight="1">
       <c r="B27" s="6" t="s">
-        <v>133</v>
+        <v>40</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>134</v>
+        <v>41</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>28</v>
@@ -1973,50 +2004,50 @@
         <v>5</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>135</v>
+        <v>43</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="K27" s="6"/>
       <c r="L27" s="6" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>138</v>
+        <v>48</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>139</v>
+        <v>49</v>
       </c>
       <c r="O27" s="6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="P27" s="6" t="s">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="Q27" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="R27" s="6"/>
       <c r="S27" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="2:19" ht="36" customHeight="1">
       <c r="B28" s="6" t="s">
-        <v>133</v>
+        <v>54</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>28</v>
@@ -2025,50 +2056,52 @@
         <v>5</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="K28" s="6"/>
       <c r="L28" s="6" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>46</v>
+        <v>127</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R28" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="S28" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="2:19" ht="36" customHeight="1">
       <c r="B29" s="6" t="s">
-        <v>133</v>
+        <v>26</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>134</v>
+        <v>27</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>28</v>
@@ -2077,50 +2110,52 @@
         <v>5</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>135</v>
+        <v>30</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>33</v>
+        <v>125</v>
       </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="N29" s="6" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="O29" s="6" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="P29" s="6" t="s">
-        <v>66</v>
+        <v>153</v>
       </c>
       <c r="Q29" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R29" s="6"/>
+        <v>37</v>
+      </c>
+      <c r="R29" s="6" t="s">
+        <v>154</v>
+      </c>
       <c r="S29" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="2:19" ht="36" customHeight="1">
       <c r="B30" s="6" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>28</v>
@@ -2129,50 +2164,52 @@
         <v>5</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>147</v>
+        <v>102</v>
       </c>
       <c r="K30" s="6"/>
       <c r="L30" s="6" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="R30" s="6"/>
+        <v>37</v>
+      </c>
+      <c r="R30" s="6" t="s">
+        <v>191</v>
+      </c>
       <c r="S30" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="2:19" ht="36" customHeight="1">
       <c r="B31" s="6" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>28</v>
@@ -2181,52 +2218,52 @@
         <v>5</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="K31" s="6"/>
       <c r="L31" s="6" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="M31" s="6" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="N31" s="6" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="O31" s="6" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="P31" s="6" t="s">
-        <v>82</v>
+        <v>149</v>
       </c>
       <c r="Q31" s="6" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="S31" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="2:19" ht="36" customHeight="1">
       <c r="B32" s="6" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>28</v>
@@ -2235,52 +2272,52 @@
         <v>5</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>136</v>
+        <v>58</v>
       </c>
       <c r="K32" s="6"/>
       <c r="L32" s="6" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>155</v>
+        <v>63</v>
       </c>
       <c r="Q32" s="6" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="S32" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="2:19" ht="36" customHeight="1">
       <c r="B33" s="6" t="s">
-        <v>26</v>
+        <v>164</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>27</v>
+        <v>165</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>28</v>
@@ -2289,52 +2326,52 @@
         <v>5</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>29</v>
+        <v>166</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>30</v>
+        <v>167</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>117</v>
+        <v>168</v>
       </c>
       <c r="K33" s="6"/>
       <c r="L33" s="6" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="N33" s="6" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="O33" s="6" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="P33" s="6" t="s">
-        <v>36</v>
+        <v>170</v>
       </c>
       <c r="Q33" s="6" t="s">
-        <v>37</v>
+        <v>171</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>182</v>
+        <v>34</v>
       </c>
       <c r="S33" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="2:19" ht="36" customHeight="1">
       <c r="B34" s="6" t="s">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>74</v>
+        <v>165</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>28</v>
@@ -2343,52 +2380,52 @@
         <v>5</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>75</v>
+        <v>166</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>76</v>
+        <v>167</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K34" s="6"/>
       <c r="L34" s="6" t="s">
-        <v>158</v>
+        <v>45</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>83</v>
+        <v>171</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="S34" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="2:19" ht="36" customHeight="1">
       <c r="B35" s="6" t="s">
-        <v>89</v>
+        <v>164</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>90</v>
+        <v>165</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>28</v>
@@ -2397,50 +2434,52 @@
         <v>5</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>91</v>
+        <v>166</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>92</v>
+        <v>167</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>52</v>
+        <v>175</v>
       </c>
       <c r="K35" s="6"/>
       <c r="L35" s="6" t="s">
-        <v>52</v>
+        <v>175</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="O35" s="6" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="P35" s="6" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="R35" s="6"/>
+        <v>171</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="S35" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="2:19" ht="36" customHeight="1">
       <c r="B36" s="6" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>28</v>
@@ -2449,50 +2488,50 @@
         <v>5</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K36" s="6"/>
       <c r="L36" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="R36" s="6"/>
       <c r="S36" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="2:19" ht="36" customHeight="1">
       <c r="B37" s="6" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>28</v>
@@ -2501,50 +2540,50 @@
         <v>5</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K37" s="6"/>
       <c r="L37" s="6" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="O37" s="6" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="P37" s="6" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="R37" s="6"/>
       <c r="S37" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="2:19" ht="36" customHeight="1">
       <c r="B38" s="6" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>28</v>
@@ -2553,50 +2592,50 @@
         <v>5</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>97</v>
+        <v>175</v>
       </c>
       <c r="K38" s="6"/>
       <c r="L38" s="6" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="R38" s="6"/>
       <c r="S38" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="2:19" ht="36" customHeight="1">
       <c r="B39" s="6" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>28</v>
@@ -2605,77 +2644,77 @@
         <v>5</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>31</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="K39" s="6"/>
       <c r="L39" s="6" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N39" s="6" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="O39" s="6" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="P39" s="6" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="R39" s="6"/>
       <c r="S39" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="2:19" ht="15.75" customHeight="1">
       <c r="B40" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C40" s="7"/>
     </row>
     <row r="41" spans="2:19" ht="15.75" customHeight="1">
       <c r="B41" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C41" s="7"/>
     </row>
-    <row r="42" spans="2:19" ht="12.75">
+    <row r="42" spans="2:19" ht="13.2">
       <c r="B42" s="2" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="9">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="2:19" ht="12.75">
+    <row r="43" spans="2:19" ht="13.2">
       <c r="B43" s="2" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="9">
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="2:19" ht="12.75">
+    <row r="44" spans="2:19" ht="13.2">
       <c r="B44" s="2" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="9">
@@ -2695,4 +2734,10 @@
   <pageSetup paperSize="9" orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" enabled="0" method="" siteId="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>